<commit_message>
feat(8140): page setup for PDF \u2014 Tabloid landscape, 0.25" margins, fit to 1 page
Certification Analysis tab now exports to a single 11x17 landscape page
with 0.25" margins. Explanation tab = portrait Letter; Certification
Requirements tab = landscape Letter (flows to 2 pages). Print area on
the pivot sheet excludes the footnote? No \u2014 includes through the
footnote row.

Verified: PDF generated at 1224x792pt (17x11in) for the matrix page.
</commit_message>
<xml_diff>
--- a/8140/8140-cert-requirements.xlsx
+++ b/8140/8140-cert-requirements.xlsx
@@ -11,7 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Certification Requirements" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Certification Analysis" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Certification Analysis'!$A$1:$BJ$52</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -2222,7 +2224,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -2350,7 +2352,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.25" footer="0.25"/>
+  <pageSetup orientation="portrait" paperSize="1" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2358,7 +2361,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3232,7 +3235,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -3240,7 +3244,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BJ52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -7970,6 +7974,8 @@
     <mergeCell ref="A1:BJ1"/>
     <mergeCell ref="T2:AL2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.1" footer="0.1"/>
+  <pageSetup orientation="landscape" paperSize="3" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(8140): finalize narrative \u2014 Master's/PhD for Advanced, 'military schooling'
- Education path updated: Bachelor's satisfies Basic/Intermediate;
  Master's or PhD now satisfies Advanced (V2.1 change from TBD).
  References 8140 Interim Education Qualification Options per V2.1.
- 'most practical route' line softened: removed 'contractors and' and
  tightened phrasing to 'may be the most practical route for anyone
  without an applicable degree or military schooling'.
- All canonical URLs verified: policy PDF via DoD CIO Library, DCWF home,
  qualification matrices, Cyber 101.

Updated DEFAULT_EXPLANATION_LINES so a fresh build produces this
narrative. Preservation logic unchanged \u2014 any hand-edits made directly
in Excel below the footnote still survive rebuilds.
</commit_message>
<xml_diff>
--- a/8140/8140-cert-requirements.xlsx
+++ b/8140/8140-cert-requirements.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Certification Analysis" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Certification Analysis'!$A$1:$BJ$59</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Certification Analysis'!$A$1:$BJ$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2219,7 +2219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BJ59"/>
+  <dimension ref="A1:BJ62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="47" customWidth="1" min="1" max="1"/>
@@ -6943,57 +6943,81 @@
     <row r="55" ht="12" customHeight="1">
       <c r="A55" s="260" t="inlineStr">
         <is>
-          <t>[PLACEHOLDER — narrative to be rewritten by Jeff.]</t>
+          <t>Governed by DoDM 8140.03 "Cyberspace Workforce Qualification and Management Program" (15 Feb 2023) — https://dodcio.defense.gov/Portals/0/Documents/Library/DoDM-8140-03.pdf. This matrix is compiled from the DoD 8140 Foundational Qualification Matrix V2.1 (effective 19 Sep 2025), published at https://www.cyber.mil/dod-workforce-innovation-directorate/dod8140/qualification-matrices.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="12" customHeight="1">
       <c r="A56" s="260" t="inlineStr">
         <is>
-          <t>Scope: certification-path qualifications only. Other paths (education, DoD training, commercial training, experience alternatives) are out of scope for this reference.</t>
+          <t>Work roles: every IT and cyber-related DoD position is mapped to one or more "work roles" — about 70 roles grouped into 7 workforce elements (Cybersecurity, IT, Cyber Enablers, Cyber Effects, Intelligence, Software Engineering, Data/AI). A single individual may hold up to 3 work roles; qualification is evaluated per role. See the DCWF at https://www.cyber.mil/dod-workforce-innovation-directorate/dod-cyber-workforce-framework. Each role has three proficiency levels (Basic, Intermediate, Advanced) — a higher-level qualification also satisfies lower levels within the same role.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="12" customHeight="1">
       <c r="A57" s="260" t="inlineStr">
         <is>
-          <t>Source: DoD 8140 Foundational Qualification Matrix V2.1 (effective 2025-09-19), via www.cyber.mil/dod-workforce-innovation-directorate/dod8140/qualification-matrices.</t>
+          <t>Qualification paths: 8140 qualification can be met via one of four "Foundational Qualification" paths — Education, DoD/Military Training, Commercial Training, or Personnel Certification — plus an "Experience" alternative for eligible personnel. This matrix shows only the Personnel Certification path, which may be the most practical route for anyone without an applicable degree or military schooling.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="12" customHeight="1">
       <c r="A58" s="260" t="inlineStr">
         <is>
-          <t>Note: CompTIA renamed CASP+ to SecurityX in 2024; both names refer to the same certification. This matrix shows it as "SecX".</t>
+          <t>Education path: Bachelor's, Master's, or PhD in Information Technology, Cybersecurity, Data Science, Information Systems, Computer Science, or Software Engineering from an ABET-accredited (abet.org) or CAE-designated (caecommunity.org) institution. Bachelor's satisfies Basic and Intermediate levels; Master's or PhD satisfies all three levels, including Advanced (a V2.1 change — previously TBD at Advanced). Degree must be within the last 5 years with documented continuous cyberspace work since. See the "8140 Interim Education Qualification Options" reference cited throughout the DoD matrix workbook for additional considerations.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="12" customHeight="1">
       <c r="A59" s="260" t="inlineStr">
         <is>
-          <t>Compiled by Jeff Krueger.</t>
+          <t>DoD / Military Training path: specific military schoolhouse courses listed per work role in the DoD 8140 Training Repository (within the same workbook linked above). Generally not accessible to government civilians or contractors unless previously completed during military service. Exception: CY 101 (40-hour online course) satisfies qualification for all Cyber Enabler work roles — https://www.cyber.mil/training/cyber-101.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="12" customHeight="1">
+      <c r="A60" s="260" t="inlineStr">
+        <is>
+          <t>Commercial Training path: commercial courses approved as 8140 qualification options. Thin option universe; most entries overlap with certifications.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="12" customHeight="1">
+      <c r="A61" s="260" t="inlineStr">
+        <is>
+          <t>Experience (alternative): available only to government civilians and military personnel. Contractors are NOT eligible for the Experience path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="12" customHeight="1">
+      <c r="A62" s="260" t="inlineStr">
+        <is>
+          <t>Compiled by Jeff Krueger. Unaffiliated with any firm, agency, or contracting office. Not legal advice.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="21">
+    <mergeCell ref="AM2:AN2"/>
+    <mergeCell ref="A62:BJ62"/>
+    <mergeCell ref="A52:BJ52"/>
+    <mergeCell ref="AZ2:BC2"/>
     <mergeCell ref="BF2:BI2"/>
-    <mergeCell ref="AO2:AW2"/>
     <mergeCell ref="A58:BJ58"/>
-    <mergeCell ref="A56:BJ56"/>
-    <mergeCell ref="AM2:AN2"/>
+    <mergeCell ref="BD2:BE2"/>
+    <mergeCell ref="A59:BJ59"/>
+    <mergeCell ref="AX2:AY2"/>
+    <mergeCell ref="A60:BJ60"/>
+    <mergeCell ref="A1:BJ1"/>
+    <mergeCell ref="A61:BJ61"/>
     <mergeCell ref="J2:O2"/>
-    <mergeCell ref="BD2:BE2"/>
-    <mergeCell ref="A55:BJ55"/>
-    <mergeCell ref="A59:BJ59"/>
-    <mergeCell ref="A57:BJ57"/>
-    <mergeCell ref="AX2:AY2"/>
     <mergeCell ref="A54:BJ54"/>
     <mergeCell ref="B2:H2"/>
-    <mergeCell ref="A52:BJ52"/>
-    <mergeCell ref="AZ2:BC2"/>
     <mergeCell ref="P2:S2"/>
-    <mergeCell ref="A1:BJ1"/>
+    <mergeCell ref="AO2:AW2"/>
+    <mergeCell ref="A56:BJ56"/>
+    <mergeCell ref="A55:BJ55"/>
+    <mergeCell ref="A57:BJ57"/>
     <mergeCell ref="T2:AL2"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
style(8140): double the explanation-block font size
Title 10->20pt, body 9->18pt, spacer 6->12pt, row heights 14/12->28/24.
Still renders on a single 11x17 page via fitToPage auto-scale.
</commit_message>
<xml_diff>
--- a/8140/8140-cert-requirements.xlsx
+++ b/8140/8140-cert-requirements.xlsx
@@ -75,12 +75,12 @@
     <font>
       <b val="1"/>
       <color rgb="FF000000"/>
-      <sz val="10"/>
+      <sz val="20"/>
     </font>
     <font>
       <i val="1"/>
       <color rgb="FF333333"/>
-      <sz val="9"/>
+      <sz val="18"/>
     </font>
   </fonts>
   <fills count="181">
@@ -6932,64 +6932,64 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="6" customHeight="1"/>
-    <row r="54" ht="14" customHeight="1">
+    <row r="53" ht="12" customHeight="1"/>
+    <row r="54" ht="28" customHeight="1">
       <c r="A54" s="259" t="inlineStr">
         <is>
           <t>DoD 8140 Cybersecurity Workforce Qualification — Personal Certification Path</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="12" customHeight="1">
+    <row r="55" ht="24" customHeight="1">
       <c r="A55" s="260" t="inlineStr">
         <is>
           <t>Governed by DoDM 8140.03 "Cyberspace Workforce Qualification and Management Program" (15 Feb 2023) — https://dodcio.defense.gov/Portals/0/Documents/Library/DoDM-8140-03.pdf. This matrix is compiled from the DoD 8140 Foundational Qualification Matrix V2.1 (effective 19 Sep 2025), published at https://www.cyber.mil/dod-workforce-innovation-directorate/dod8140/qualification-matrices.</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="12" customHeight="1">
+    <row r="56" ht="24" customHeight="1">
       <c r="A56" s="260" t="inlineStr">
         <is>
           <t>Work roles: every IT and cyber-related DoD position is mapped to one or more "work roles" — about 70 roles grouped into 7 workforce elements (Cybersecurity, IT, Cyber Enablers, Cyber Effects, Intelligence, Software Engineering, Data/AI). A single individual may hold up to 3 work roles; qualification is evaluated per role. See the DCWF at https://www.cyber.mil/dod-workforce-innovation-directorate/dod-cyber-workforce-framework. Each role has three proficiency levels (Basic, Intermediate, Advanced) — a higher-level qualification also satisfies lower levels within the same role.</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="12" customHeight="1">
+    <row r="57" ht="24" customHeight="1">
       <c r="A57" s="260" t="inlineStr">
         <is>
           <t>Qualification paths: 8140 qualification can be met via one of four "Foundational Qualification" paths — Education, DoD/Military Training, Commercial Training, or Personnel Certification — plus an "Experience" alternative for eligible personnel. This matrix shows only the Personnel Certification path, which may be the most practical route for anyone without an applicable degree or military schooling.</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="12" customHeight="1">
+    <row r="58" ht="24" customHeight="1">
       <c r="A58" s="260" t="inlineStr">
         <is>
           <t>Education path: Bachelor's, Master's, or PhD in Information Technology, Cybersecurity, Data Science, Information Systems, Computer Science, or Software Engineering from an ABET-accredited (abet.org) or CAE-designated (caecommunity.org) institution. Bachelor's satisfies Basic and Intermediate levels; Master's or PhD satisfies all three levels, including Advanced (a V2.1 change — previously TBD at Advanced). Degree must be within the last 5 years with documented continuous cyberspace work since. See the "8140 Interim Education Qualification Options" reference cited throughout the DoD matrix workbook for additional considerations.</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="12" customHeight="1">
+    <row r="59" ht="24" customHeight="1">
       <c r="A59" s="260" t="inlineStr">
         <is>
           <t>DoD / Military Training path: specific military schoolhouse courses listed per work role in the DoD 8140 Training Repository (within the same workbook linked above). Generally not accessible to government civilians or contractors unless previously completed during military service. Exception: CY 101 (40-hour online course) satisfies qualification for all Cyber Enabler work roles — https://www.cyber.mil/training/cyber-101.</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="12" customHeight="1">
+    <row r="60" ht="24" customHeight="1">
       <c r="A60" s="260" t="inlineStr">
         <is>
           <t>Commercial Training path: commercial courses approved as 8140 qualification options. Thin option universe; most entries overlap with certifications.</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="12" customHeight="1">
+    <row r="61" ht="24" customHeight="1">
       <c r="A61" s="260" t="inlineStr">
         <is>
           <t>Experience (alternative): available only to government civilians and military personnel. Contractors are NOT eligible for the Experience path.</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="12" customHeight="1">
+    <row r="62" ht="24" customHeight="1">
       <c r="A62" s="260" t="inlineStr">
         <is>
           <t>Compiled by Jeff Krueger. Unaffiliated with any firm, agency, or contracting office. Not legal advice.</t>

</xml_diff>

<commit_message>
style(8140): narrative fonts 14pt title / 12pt body; per-row height sizing
Row heights now estimated from wrapped-line count (approx 230 chars per
visual line at merged A:BJ width, with 0.88 word-wrap efficiency, 1.35x
line-height). Rows size from 22pt (single-line entries) up to 70pt (the
longer Education paragraph). No clipping; no wasted vertical space on
short lines. Still one 11x17 landscape page.
</commit_message>
<xml_diff>
--- a/8140/8140-cert-requirements.xlsx
+++ b/8140/8140-cert-requirements.xlsx
@@ -75,12 +75,12 @@
     <font>
       <b val="1"/>
       <color rgb="FF000000"/>
-      <sz val="20"/>
+      <sz val="14"/>
     </font>
     <font>
       <i val="1"/>
       <color rgb="FF333333"/>
-      <sz val="18"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="181">
@@ -6932,64 +6932,64 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="12" customHeight="1"/>
-    <row r="54" ht="28" customHeight="1">
+    <row r="53" ht="8" customHeight="1"/>
+    <row r="54" ht="24" customHeight="1">
       <c r="A54" s="259" t="inlineStr">
         <is>
           <t>DoD 8140 Cybersecurity Workforce Qualification — Personal Certification Path</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="24" customHeight="1">
+    <row r="55" ht="38" customHeight="1">
       <c r="A55" s="260" t="inlineStr">
         <is>
           <t>Governed by DoDM 8140.03 "Cyberspace Workforce Qualification and Management Program" (15 Feb 2023) — https://dodcio.defense.gov/Portals/0/Documents/Library/DoDM-8140-03.pdf. This matrix is compiled from the DoD 8140 Foundational Qualification Matrix V2.1 (effective 19 Sep 2025), published at https://www.cyber.mil/dod-workforce-innovation-directorate/dod8140/qualification-matrices.</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="24" customHeight="1">
+    <row r="56" ht="54" customHeight="1">
       <c r="A56" s="260" t="inlineStr">
         <is>
           <t>Work roles: every IT and cyber-related DoD position is mapped to one or more "work roles" — about 70 roles grouped into 7 workforce elements (Cybersecurity, IT, Cyber Enablers, Cyber Effects, Intelligence, Software Engineering, Data/AI). A single individual may hold up to 3 work roles; qualification is evaluated per role. See the DCWF at https://www.cyber.mil/dod-workforce-innovation-directorate/dod-cyber-workforce-framework. Each role has three proficiency levels (Basic, Intermediate, Advanced) — a higher-level qualification also satisfies lower levels within the same role.</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="24" customHeight="1">
+    <row r="57" ht="38" customHeight="1">
       <c r="A57" s="260" t="inlineStr">
         <is>
           <t>Qualification paths: 8140 qualification can be met via one of four "Foundational Qualification" paths — Education, DoD/Military Training, Commercial Training, or Personnel Certification — plus an "Experience" alternative for eligible personnel. This matrix shows only the Personnel Certification path, which may be the most practical route for anyone without an applicable degree or military schooling.</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="24" customHeight="1">
+    <row r="58" ht="70" customHeight="1">
       <c r="A58" s="260" t="inlineStr">
         <is>
           <t>Education path: Bachelor's, Master's, or PhD in Information Technology, Cybersecurity, Data Science, Information Systems, Computer Science, or Software Engineering from an ABET-accredited (abet.org) or CAE-designated (caecommunity.org) institution. Bachelor's satisfies Basic and Intermediate levels; Master's or PhD satisfies all three levels, including Advanced (a V2.1 change — previously TBD at Advanced). Degree must be within the last 5 years with documented continuous cyberspace work since. See the "8140 Interim Education Qualification Options" reference cited throughout the DoD matrix workbook for additional considerations.</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="24" customHeight="1">
+    <row r="59" ht="54" customHeight="1">
       <c r="A59" s="260" t="inlineStr">
         <is>
           <t>DoD / Military Training path: specific military schoolhouse courses listed per work role in the DoD 8140 Training Repository (within the same workbook linked above). Generally not accessible to government civilians or contractors unless previously completed during military service. Exception: CY 101 (40-hour online course) satisfies qualification for all Cyber Enabler work roles — https://www.cyber.mil/training/cyber-101.</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="24" customHeight="1">
+    <row r="60" ht="22" customHeight="1">
       <c r="A60" s="260" t="inlineStr">
         <is>
           <t>Commercial Training path: commercial courses approved as 8140 qualification options. Thin option universe; most entries overlap with certifications.</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="24" customHeight="1">
+    <row r="61" ht="22" customHeight="1">
       <c r="A61" s="260" t="inlineStr">
         <is>
           <t>Experience (alternative): available only to government civilians and military personnel. Contractors are NOT eligible for the Experience path.</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="24" customHeight="1">
+    <row r="62" ht="22" customHeight="1">
       <c r="A62" s="260" t="inlineStr">
         <is>
           <t>Compiled by Jeff Krueger. Unaffiliated with any firm, agency, or contracting office. Not legal advice.</t>

</xml_diff>